<commit_message>
p226 parts pretty names
</commit_message>
<xml_diff>
--- a/changes/p226_parts.xlsx
+++ b/changes/p226_parts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WhyTh\Documents\GitHub\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B59BD4CF-47AA-45B8-9E14-D8CC814CDAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A385D71-6635-4583-B1B7-38B5427C9F4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="123">
   <si>
     <t>new</t>
   </si>
@@ -270,6 +270,141 @@
   </si>
   <si>
     <t>suppressors_inc_p226_5inch_threaded_9x19_barrel</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 Standard</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226R</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 MK25</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 Elite</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 Standard 9x19</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 Elite DRD Optics Cut 9x19</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 Elite 9x19</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 PRO-CUT 9x19</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 RXP 9x19</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 MK25 9x19</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P229 Standard 9x19</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P229 Elite 9x19</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P229 Elite Legacy 9x19</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P229 Legacy 9x19</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P229 RXP 9x19</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 Flush Sight Plate</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 Sight Plate</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P229 Flush Sight Plate</t>
+  </si>
+  <si>
+    <t>D&amp;L Precision P226/P229 DRD Filler Plate</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P-Series OEM</t>
+  </si>
+  <si>
+    <t>LaseVex SIC P-Series</t>
+  </si>
+  <si>
+    <t>GoForce SIC P-Series Drive Ledge</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 Standard Two-Piece</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 Standard Two-Piece Magwell</t>
+  </si>
+  <si>
+    <t>Rogue P226 Smooth Hardwood</t>
+  </si>
+  <si>
+    <t>Metrik Precision SIC P-Series Skeletonized</t>
+  </si>
+  <si>
+    <t>ASHGUNS SIC P-Series Adjustable Straight</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 OEM</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P229 OEM</t>
+  </si>
+  <si>
+    <t>LaseVex P226 Green Laser</t>
+  </si>
+  <si>
+    <t>LaseVex P229 Green Laser</t>
+  </si>
+  <si>
+    <t>ASHGUNS SIC P-Series Modern Heritage Commander</t>
+  </si>
+  <si>
+    <t>Ravaryn Arms SIC P-Series Skeletonized</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ravaryn Arms SIC P-Series Extended </t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 9x19 15R</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 Mag</t>
+  </si>
+  <si>
+    <t>Nexa Tactical P226 4R Extension</t>
+  </si>
+  <si>
+    <t>Everetts Machining SIC 226/229 Duty</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P229 OEM 3.9" 9x19</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P229 OEM 4.4" Threaded 9x19</t>
+  </si>
+  <si>
+    <t>VAL-BOR P229 4.4" Threaded Match Grade 9x19</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 OEM 4.4" 9x19</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P226 OEM 5" 9x19</t>
+  </si>
+  <si>
+    <t>Suppressors Inc. P226 5" Threaded 9x19</t>
+  </si>
+  <si>
+    <t>sic_sturmer_p_series_oem_slide_release</t>
   </si>
 </sst>
 </file>
@@ -587,7 +722,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P64"/>
+  <dimension ref="A1:P65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -651,8 +786,11 @@
       <c r="B4" t="s">
         <v>17</v>
       </c>
+      <c r="C4" t="s">
+        <v>78</v>
+      </c>
       <c r="P4">
-        <f t="shared" ref="P4:P64" si="0">D4-E4*20-F4*0.8-G4*0.6-I4*10+J4*15+O4/200-N4*5</f>
+        <f>D4-E4*20-F4*0.8-G4*0.6-I4*10+J4*15+O4/200-N4*5</f>
         <v>0</v>
       </c>
     </row>
@@ -660,8 +798,11 @@
       <c r="B5" t="s">
         <v>18</v>
       </c>
+      <c r="C5" t="s">
+        <v>79</v>
+      </c>
       <c r="P5">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="P5:P65" si="0">D5-E5*20-F5*0.8-G5*0.6-I5*10+J5*15+O5/200-N5*5</f>
         <v>0</v>
       </c>
     </row>
@@ -669,6 +810,9 @@
       <c r="B6" t="s">
         <v>19</v>
       </c>
+      <c r="C6" t="s">
+        <v>80</v>
+      </c>
       <c r="P6">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -678,6 +822,9 @@
       <c r="B7" t="s">
         <v>20</v>
       </c>
+      <c r="C7" t="s">
+        <v>81</v>
+      </c>
       <c r="P7">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -692,6 +839,9 @@
       <c r="B9" t="s">
         <v>22</v>
       </c>
+      <c r="C9" t="s">
+        <v>82</v>
+      </c>
       <c r="P9">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -701,6 +851,9 @@
       <c r="B10" t="s">
         <v>23</v>
       </c>
+      <c r="C10" t="s">
+        <v>83</v>
+      </c>
       <c r="P10">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -710,6 +863,9 @@
       <c r="B11" t="s">
         <v>24</v>
       </c>
+      <c r="C11" t="s">
+        <v>84</v>
+      </c>
       <c r="P11">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -719,6 +875,9 @@
       <c r="B12" t="s">
         <v>25</v>
       </c>
+      <c r="C12" t="s">
+        <v>85</v>
+      </c>
       <c r="P12">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -728,6 +887,9 @@
       <c r="B13" t="s">
         <v>26</v>
       </c>
+      <c r="C13" t="s">
+        <v>86</v>
+      </c>
       <c r="P13">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -737,6 +899,9 @@
       <c r="B14" t="s">
         <v>27</v>
       </c>
+      <c r="C14" t="s">
+        <v>87</v>
+      </c>
       <c r="P14">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -746,6 +911,9 @@
       <c r="B15" t="s">
         <v>28</v>
       </c>
+      <c r="C15" t="s">
+        <v>88</v>
+      </c>
       <c r="P15">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -755,6 +923,9 @@
       <c r="B16" t="s">
         <v>29</v>
       </c>
+      <c r="C16" t="s">
+        <v>89</v>
+      </c>
       <c r="P16">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -764,6 +935,9 @@
       <c r="B17" t="s">
         <v>30</v>
       </c>
+      <c r="C17" t="s">
+        <v>90</v>
+      </c>
       <c r="P17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -773,6 +947,9 @@
       <c r="B18" t="s">
         <v>31</v>
       </c>
+      <c r="C18" t="s">
+        <v>91</v>
+      </c>
       <c r="P18">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -782,6 +959,9 @@
       <c r="B19" t="s">
         <v>32</v>
       </c>
+      <c r="C19" t="s">
+        <v>92</v>
+      </c>
       <c r="P19">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -800,11 +980,17 @@
       <c r="B21" t="s">
         <v>34</v>
       </c>
+      <c r="C21" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>35</v>
       </c>
+      <c r="C22" t="s">
+        <v>94</v>
+      </c>
       <c r="P22">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -814,6 +1000,9 @@
       <c r="B23" t="s">
         <v>36</v>
       </c>
+      <c r="C23" t="s">
+        <v>95</v>
+      </c>
       <c r="P23">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -823,6 +1012,9 @@
       <c r="B24" t="s">
         <v>37</v>
       </c>
+      <c r="C24" t="s">
+        <v>96</v>
+      </c>
       <c r="P24">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -832,6 +1024,9 @@
       <c r="B25" t="s">
         <v>38</v>
       </c>
+      <c r="C25" t="s">
+        <v>93</v>
+      </c>
       <c r="P25">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -841,6 +1036,9 @@
       <c r="B26" t="s">
         <v>39</v>
       </c>
+      <c r="C26" t="s">
+        <v>94</v>
+      </c>
       <c r="P26">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -855,6 +1053,9 @@
       <c r="B28" t="s">
         <v>41</v>
       </c>
+      <c r="C28" t="s">
+        <v>97</v>
+      </c>
       <c r="P28">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -864,6 +1065,9 @@
       <c r="B29" t="s">
         <v>42</v>
       </c>
+      <c r="C29" t="s">
+        <v>98</v>
+      </c>
       <c r="P29">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -873,6 +1077,9 @@
       <c r="B30" t="s">
         <v>43</v>
       </c>
+      <c r="C30" t="s">
+        <v>99</v>
+      </c>
       <c r="P30">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -891,6 +1098,9 @@
       <c r="B32" t="s">
         <v>45</v>
       </c>
+      <c r="C32" t="s">
+        <v>100</v>
+      </c>
       <c r="P32">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -900,6 +1110,9 @@
       <c r="B33" t="s">
         <v>46</v>
       </c>
+      <c r="C33" t="s">
+        <v>101</v>
+      </c>
       <c r="P33">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -909,6 +1122,9 @@
       <c r="B34" t="s">
         <v>47</v>
       </c>
+      <c r="C34" t="s">
+        <v>102</v>
+      </c>
       <c r="P34">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -923,6 +1139,9 @@
       <c r="B36" t="s">
         <v>49</v>
       </c>
+      <c r="C36" t="s">
+        <v>97</v>
+      </c>
       <c r="P36">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -932,6 +1151,9 @@
       <c r="B37" t="s">
         <v>50</v>
       </c>
+      <c r="C37" t="s">
+        <v>103</v>
+      </c>
       <c r="P37">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -941,6 +1163,9 @@
       <c r="B38" t="s">
         <v>51</v>
       </c>
+      <c r="C38" t="s">
+        <v>104</v>
+      </c>
       <c r="P38">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -959,6 +1184,9 @@
       <c r="B40" t="s">
         <v>53</v>
       </c>
+      <c r="C40" t="s">
+        <v>105</v>
+      </c>
       <c r="P40">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -968,6 +1196,9 @@
       <c r="B41" t="s">
         <v>54</v>
       </c>
+      <c r="C41" t="s">
+        <v>106</v>
+      </c>
       <c r="P41">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -977,6 +1208,9 @@
       <c r="B42" t="s">
         <v>55</v>
       </c>
+      <c r="C42" t="s">
+        <v>107</v>
+      </c>
       <c r="P42">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -986,6 +1220,9 @@
       <c r="B43" t="s">
         <v>56</v>
       </c>
+      <c r="C43" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
@@ -1000,6 +1237,9 @@
       <c r="B45" t="s">
         <v>58</v>
       </c>
+      <c r="C45" t="s">
+        <v>97</v>
+      </c>
       <c r="P45">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1009,6 +1249,9 @@
       <c r="B46" t="s">
         <v>59</v>
       </c>
+      <c r="C46" t="s">
+        <v>109</v>
+      </c>
       <c r="P46">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1018,6 +1261,9 @@
       <c r="B47" t="s">
         <v>60</v>
       </c>
+      <c r="C47" t="s">
+        <v>110</v>
+      </c>
       <c r="P47">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1032,6 +1278,9 @@
       <c r="B49" t="s">
         <v>62</v>
       </c>
+      <c r="C49" t="s">
+        <v>97</v>
+      </c>
       <c r="P49">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1041,6 +1290,9 @@
       <c r="B50" t="s">
         <v>63</v>
       </c>
+      <c r="C50" t="s">
+        <v>111</v>
+      </c>
       <c r="P50">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1059,6 +1311,9 @@
       <c r="B52" t="s">
         <v>65</v>
       </c>
+      <c r="C52" t="s">
+        <v>112</v>
+      </c>
       <c r="P52">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1068,6 +1323,9 @@
       <c r="B53" t="s">
         <v>66</v>
       </c>
+      <c r="C53" t="s">
+        <v>113</v>
+      </c>
       <c r="P53">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1077,6 +1335,9 @@
       <c r="B54" t="s">
         <v>67</v>
       </c>
+      <c r="C54" t="s">
+        <v>114</v>
+      </c>
       <c r="P54">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1091,6 +1352,9 @@
       <c r="B56" t="s">
         <v>69</v>
       </c>
+      <c r="C56" t="s">
+        <v>97</v>
+      </c>
       <c r="P56">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1098,30 +1362,39 @@
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
+        <v>122</v>
+      </c>
+      <c r="C57" t="s">
+        <v>97</v>
+      </c>
+      <c r="P57">
+        <f>D57-E57*20-F57*0.8-G57*0.6-I57*10+J57*15+O57/200-N57*5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B58" t="s">
         <v>70</v>
       </c>
-      <c r="P57">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+      <c r="C58" t="s">
+        <v>115</v>
+      </c>
+      <c r="P58">
+        <f>D58-E58*20-F58*0.8-G58*0.6-I58*10+J58*15+O58/200-N58*5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
         <v>71</v>
-      </c>
-    </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B59" t="s">
-        <v>72</v>
-      </c>
-      <c r="P59">
-        <f t="shared" si="0"/>
-        <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
-        <v>73</v>
+        <v>72</v>
+      </c>
+      <c r="C60" t="s">
+        <v>116</v>
       </c>
       <c r="P60">
         <f t="shared" si="0"/>
@@ -1130,7 +1403,10 @@
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
-        <v>74</v>
+        <v>73</v>
+      </c>
+      <c r="C61" t="s">
+        <v>117</v>
       </c>
       <c r="P61">
         <f t="shared" si="0"/>
@@ -1139,7 +1415,10 @@
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
-        <v>75</v>
+        <v>74</v>
+      </c>
+      <c r="C62" t="s">
+        <v>118</v>
       </c>
       <c r="P62">
         <f t="shared" si="0"/>
@@ -1148,7 +1427,10 @@
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>76</v>
+        <v>75</v>
+      </c>
+      <c r="C63" t="s">
+        <v>119</v>
       </c>
       <c r="P63">
         <f t="shared" si="0"/>
@@ -1157,9 +1439,24 @@
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
+        <v>76</v>
+      </c>
+      <c r="C64" t="s">
+        <v>120</v>
+      </c>
+      <c r="P64">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
         <v>77</v>
       </c>
-      <c r="P64">
+      <c r="C65" t="s">
+        <v>121</v>
+      </c>
+      <c r="P65">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
p226 tweaks part one
Guys. I Fucked Up.
</commit_message>
<xml_diff>
--- a/changes/p226_parts.xlsx
+++ b/changes/p226_parts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WhyTh\Documents\GitHub\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{858F4307-DF3C-4327-A15A-1D98443F7B1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59A14F58-DDD8-407B-94D4-9225623F39C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -392,19 +392,19 @@
     <t>Sic Stürmer P229 OEM 4.4" Threaded 9x19</t>
   </si>
   <si>
-    <t>VAL-BOR P229 4.4" Threaded Match Grade 9x19</t>
-  </si>
-  <si>
     <t>Sic Stürmer P226 OEM 4.4" 9x19</t>
   </si>
   <si>
     <t>sic_sturmer_p_series_oem_slide_release</t>
   </si>
   <si>
-    <t>Suppressors Inc. P226 5" Threaded Match Grade 9x19</t>
-  </si>
-  <si>
     <t>Sic Stürmer P226 OEM 5" Threaded 9x19</t>
+  </si>
+  <si>
+    <t>VAL-BOR P229 4.4" Threaded 9x19</t>
+  </si>
+  <si>
+    <t>Suppressors Inc. P226 5" Threaded 9x19</t>
   </si>
 </sst>
 </file>
@@ -934,7 +934,7 @@
         <v>83</v>
       </c>
       <c r="D10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10">
         <v>0.23</v>
@@ -950,7 +950,7 @@
       </c>
       <c r="P10">
         <f t="shared" si="0"/>
-        <v>0.19999999999999951</v>
+        <v>-0.80000000000000049</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
@@ -988,7 +988,7 @@
         <v>85</v>
       </c>
       <c r="D12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E12">
         <v>0.2</v>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="P12">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
@@ -1015,7 +1015,7 @@
         <v>86</v>
       </c>
       <c r="D13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13">
         <v>0.19</v>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="P13">
         <f t="shared" si="0"/>
-        <v>0.6000000000000002</v>
+        <v>-0.3999999999999998</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
@@ -1177,7 +1177,7 @@
         <v>92</v>
       </c>
       <c r="D19">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E19">
         <v>0.18</v>
@@ -1193,7 +1193,7 @@
       </c>
       <c r="P19">
         <f t="shared" si="0"/>
-        <v>0.40000000000000036</v>
+        <v>-0.59999999999999964</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
@@ -1804,6 +1804,9 @@
       <c r="E52">
         <v>0.23</v>
       </c>
+      <c r="H52">
+        <v>15</v>
+      </c>
       <c r="N52">
         <v>0</v>
       </c>
@@ -1882,7 +1885,7 @@
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C57" t="s">
         <v>97</v>
@@ -1947,10 +1950,10 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F60">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G60">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I60">
         <v>0.1</v>
@@ -1966,7 +1969,7 @@
       </c>
       <c r="P60">
         <f t="shared" si="0"/>
-        <v>-4.0999999999999996</v>
+        <v>-5.5</v>
       </c>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
@@ -1983,10 +1986,10 @@
         <v>0.09</v>
       </c>
       <c r="F61">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I61">
         <v>7.0000000000000007E-2</v>
@@ -1999,7 +2002,7 @@
       </c>
       <c r="P61">
         <f t="shared" si="0"/>
-        <v>-3.5</v>
+        <v>-5.7</v>
       </c>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
@@ -2007,7 +2010,7 @@
         <v>74</v>
       </c>
       <c r="C62" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D62">
         <v>-1</v>
@@ -2016,10 +2019,10 @@
         <v>0.1</v>
       </c>
       <c r="F62">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G62">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I62">
         <v>0.05</v>
@@ -2032,7 +2035,7 @@
       </c>
       <c r="P62">
         <f t="shared" si="0"/>
-        <v>-3.5</v>
+        <v>-6.3</v>
       </c>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
@@ -2040,7 +2043,7 @@
         <v>75</v>
       </c>
       <c r="C63" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D63">
         <v>0</v>
@@ -2073,7 +2076,7 @@
         <v>76</v>
       </c>
       <c r="C64" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D64">
         <v>-2</v>
@@ -2109,7 +2112,7 @@
         <v>77</v>
       </c>
       <c r="C65" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D65">
         <v>-2</v>

</xml_diff>

<commit_message>
p226 tweaks part two
- add p226 to bipods.csv, disallow mounting
- decrease base ergo from 65 -> 60
- misc. price tweaks
</commit_message>
<xml_diff>
--- a/changes/p226_parts.xlsx
+++ b/changes/p226_parts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WhyTh\Documents\GitHub\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59A14F58-DDD8-407B-94D4-9225623F39C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22D20EAF-26F9-436D-A5EC-0346D52B13D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1257,7 +1257,7 @@
         <v>0.03</v>
       </c>
       <c r="N23">
-        <v>225</v>
+        <v>150</v>
       </c>
       <c r="P23">
         <f t="shared" si="0"/>
@@ -1320,7 +1320,7 @@
         <v>0.04</v>
       </c>
       <c r="N26">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="P26">
         <f t="shared" si="0"/>

</xml_diff>